<commit_message>
Pick up updated OGZ temperature data and fix stale cache
The GKL protection temperature spreadsheet was updated with new values.
Also make load_ogz_data()'s cache key include the file's mtime, so a
running app (e.g. on Streamlit Cloud) picks up future edits to the
spreadsheet without needing a manual restart.
</commit_message>
<xml_diff>
--- a/температура с ОГЗ.xlsx
+++ b/температура с ОГЗ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YandexDisk\02_PROJECT\Python\steel\Steel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{68567220-FBFD-4520-AB62-F478E8CB8D38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71609E93-A3D3-494A-B5FD-19737B461C96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CF9B73C0-209F-4FC5-92E1-844AEABB6AA9}"/>
   </bookViews>
@@ -442,7 +442,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAC3D793-1B4D-4106-BC8E-E67CFBC449AE}">
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -478,13 +478,13 @@
         <v>90</v>
       </c>
       <c r="B3">
-        <v>20.526</v>
+        <v>20.675999999999998</v>
       </c>
       <c r="C3">
-        <v>20.071000000000002</v>
+        <v>20.350999999999999</v>
       </c>
       <c r="D3">
-        <v>22.210999999999999</v>
+        <v>23.224</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -492,755 +492,811 @@
         <v>120</v>
       </c>
       <c r="B4">
-        <v>20.925000000000001</v>
+        <v>21.058</v>
       </c>
       <c r="C4">
-        <v>20.204000000000001</v>
+        <v>20.721</v>
       </c>
       <c r="D4">
-        <v>23.873999999999999</v>
+        <v>24.882000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>141.03</v>
+        <v>141.85</v>
       </c>
       <c r="B5">
-        <v>21.274999999999999</v>
+        <v>21.419</v>
       </c>
       <c r="C5">
-        <v>20.343</v>
+        <v>21.077999999999999</v>
       </c>
       <c r="D5">
-        <v>25.34</v>
+        <v>26.443999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>162.07</v>
+        <v>163.69999999999999</v>
       </c>
       <c r="B6">
-        <v>21.702999999999999</v>
+        <v>21.872</v>
       </c>
       <c r="C6">
-        <v>20.535</v>
+        <v>21.545999999999999</v>
       </c>
       <c r="D6">
-        <v>27.146999999999998</v>
+        <v>28.401</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>200.59</v>
+        <v>203.04</v>
       </c>
       <c r="B7">
-        <v>22.766999999999999</v>
+        <v>23.016999999999999</v>
       </c>
       <c r="C7">
-        <v>21.131</v>
+        <v>22.866</v>
       </c>
       <c r="D7">
-        <v>31.603999999999999</v>
+        <v>33.222000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>246.55</v>
+        <v>250.18</v>
       </c>
       <c r="B8">
-        <v>24.417000000000002</v>
+        <v>24.899000000000001</v>
       </c>
       <c r="C8">
-        <v>22.283000000000001</v>
+        <v>25.359000000000002</v>
       </c>
       <c r="D8">
-        <v>38.351999999999997</v>
+        <v>40.697000000000003</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>298.08999999999997</v>
+        <v>303.41000000000003</v>
       </c>
       <c r="B9">
-        <v>26.702000000000002</v>
+        <v>27.706</v>
       </c>
       <c r="C9">
-        <v>24.213000000000001</v>
+        <v>29.556000000000001</v>
       </c>
       <c r="D9">
-        <v>47.338000000000001</v>
+        <v>50.960999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>354.64</v>
+        <v>362.16</v>
       </c>
       <c r="B10">
-        <v>29.67</v>
+        <v>31.666</v>
       </c>
       <c r="C10">
-        <v>27.134</v>
+        <v>35.996000000000002</v>
       </c>
       <c r="D10">
-        <v>58.411000000000001</v>
+        <v>64.06</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>415.46</v>
+        <v>425.82</v>
       </c>
       <c r="B11">
-        <v>33.326999999999998</v>
+        <v>36.968000000000004</v>
       </c>
       <c r="C11">
-        <v>31.166</v>
+        <v>45.037999999999997</v>
       </c>
       <c r="D11">
-        <v>71.221999999999994</v>
+        <v>79.831000000000003</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>480.16</v>
+        <v>494.32</v>
       </c>
       <c r="B12">
-        <v>37.597999999999999</v>
+        <v>43.142000000000003</v>
       </c>
       <c r="C12">
-        <v>36.381999999999998</v>
+        <v>54.982999999999997</v>
       </c>
       <c r="D12">
-        <v>85.015000000000001</v>
+        <v>96.956000000000003</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>594.33000000000004</v>
+        <v>609.97</v>
       </c>
       <c r="B13">
-        <v>46.307000000000002</v>
+        <v>56.963999999999999</v>
       </c>
       <c r="C13">
-        <v>47.505000000000003</v>
+        <v>78.697999999999993</v>
       </c>
       <c r="D13">
-        <v>110.22</v>
+        <v>129.21</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>646.78</v>
+        <v>672.85</v>
       </c>
       <c r="B14">
-        <v>50.5</v>
+        <v>64.855000000000004</v>
       </c>
       <c r="C14">
-        <v>53.024999999999999</v>
+        <v>91.531000000000006</v>
       </c>
       <c r="D14">
-        <v>121.65</v>
+        <v>146.56</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>699.23</v>
+        <v>735.73</v>
       </c>
       <c r="B15">
-        <v>54.857999999999997</v>
+        <v>73.323999999999998</v>
       </c>
       <c r="C15">
-        <v>58.823</v>
+        <v>105.18</v>
       </c>
       <c r="D15">
-        <v>132.94999999999999</v>
+        <v>164.03</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>792.43</v>
+        <v>841.95</v>
       </c>
       <c r="B16">
-        <v>62.99</v>
+        <v>88.438999999999993</v>
       </c>
       <c r="C16">
-        <v>69.757000000000005</v>
+        <v>128.24</v>
       </c>
       <c r="D16">
-        <v>152.19</v>
+        <v>192.67</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>923.74</v>
+        <v>991.17</v>
       </c>
       <c r="B17">
-        <v>75.064999999999998</v>
+        <v>110.63</v>
       </c>
       <c r="C17">
-        <v>85.242999999999995</v>
+        <v>160.22</v>
       </c>
       <c r="D17">
-        <v>178.56</v>
+        <v>230.87</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>983.86</v>
+        <v>1149.4000000000001</v>
       </c>
       <c r="B18">
-        <v>80.724000000000004</v>
+        <v>138.05000000000001</v>
       </c>
       <c r="C18">
-        <v>92.400999999999996</v>
+        <v>201.2</v>
       </c>
       <c r="D18">
-        <v>190.47</v>
+        <v>274.45999999999998</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>1044</v>
+        <v>1220.4000000000001</v>
       </c>
       <c r="B19">
-        <v>86.474000000000004</v>
+        <v>150.69999999999999</v>
       </c>
       <c r="C19">
-        <v>99.590999999999994</v>
+        <v>219.51</v>
       </c>
       <c r="D19">
-        <v>202.12</v>
+        <v>293.92</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>1104.0999999999999</v>
+        <v>1291.4000000000001</v>
       </c>
       <c r="B20">
-        <v>92.286000000000001</v>
+        <v>163.59</v>
       </c>
       <c r="C20">
-        <v>106.78</v>
+        <v>237.63</v>
       </c>
       <c r="D20">
-        <v>213.47</v>
+        <v>313.10000000000002</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>1226.5999999999999</v>
+        <v>1451.2</v>
       </c>
       <c r="B21">
-        <v>104.21</v>
+        <v>193</v>
       </c>
       <c r="C21">
-        <v>121.2</v>
+        <v>276.94</v>
       </c>
       <c r="D21">
-        <v>235.18</v>
+        <v>354.08</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>1349.1</v>
+        <v>1611</v>
       </c>
       <c r="B22">
-        <v>116.08</v>
+        <v>222.12</v>
       </c>
       <c r="C22">
-        <v>135.22</v>
+        <v>313.97000000000003</v>
       </c>
       <c r="D22">
-        <v>255.49</v>
+        <v>392.35</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>1490.1</v>
+        <v>1804.6</v>
       </c>
       <c r="B23">
-        <v>129.55000000000001</v>
+        <v>257.02</v>
       </c>
       <c r="C23">
-        <v>150.65</v>
+        <v>356.81</v>
       </c>
       <c r="D23">
-        <v>277.08</v>
+        <v>435.26</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>1640</v>
+        <v>1998.1</v>
       </c>
       <c r="B24">
-        <v>143.52000000000001</v>
+        <v>291.11</v>
       </c>
       <c r="C24">
-        <v>166.14</v>
+        <v>396.97</v>
       </c>
       <c r="D24">
-        <v>298.12</v>
+        <v>474.69</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>1799.1</v>
+        <v>2198.9</v>
       </c>
       <c r="B25">
-        <v>157.83000000000001</v>
+        <v>325.41000000000003</v>
       </c>
       <c r="C25">
-        <v>181.48</v>
+        <v>435.81</v>
       </c>
       <c r="D25">
-        <v>318.45</v>
+        <v>512.05999999999995</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>1965.6</v>
+        <v>2401</v>
       </c>
       <c r="B26">
-        <v>172.18</v>
+        <v>358.73</v>
       </c>
       <c r="C26">
-        <v>196.31</v>
+        <v>472.19</v>
       </c>
       <c r="D26">
-        <v>337.7</v>
+        <v>546.41999999999996</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>2139.1999999999998</v>
+        <v>2603.1</v>
       </c>
       <c r="B27">
-        <v>186.39</v>
+        <v>390.79</v>
       </c>
       <c r="C27">
-        <v>210.48</v>
+        <v>506.02</v>
       </c>
       <c r="D27">
-        <v>355.77</v>
+        <v>577.80999999999995</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>2319.1</v>
+        <v>2805.2</v>
       </c>
       <c r="B28">
-        <v>200.31</v>
+        <v>421.55</v>
       </c>
       <c r="C28">
-        <v>223.85</v>
+        <v>537.46</v>
       </c>
       <c r="D28">
-        <v>372.56</v>
+        <v>606.5</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>2504.6999999999998</v>
+        <v>3007.3</v>
       </c>
       <c r="B29">
-        <v>213.77</v>
+        <v>450.98</v>
       </c>
       <c r="C29">
-        <v>236.32</v>
+        <v>566.65</v>
       </c>
       <c r="D29">
-        <v>388.03</v>
+        <v>632.61</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>2695.2</v>
+        <v>3209.4</v>
       </c>
       <c r="B30">
-        <v>226.69</v>
+        <v>479.07</v>
       </c>
       <c r="C30">
-        <v>247.86</v>
+        <v>593.72</v>
       </c>
       <c r="D30">
-        <v>402.18</v>
+        <v>656.24</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>2890.2</v>
+        <v>3411.5</v>
       </c>
       <c r="B31">
-        <v>238.99</v>
+        <v>505.82</v>
       </c>
       <c r="C31">
-        <v>258.45999999999998</v>
+        <v>618.69000000000005</v>
       </c>
       <c r="D31">
-        <v>415.06</v>
+        <v>677.43</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>3089.1</v>
+        <v>3613.6</v>
       </c>
       <c r="B32">
-        <v>250.63</v>
+        <v>530.62</v>
       </c>
       <c r="C32">
-        <v>268.13</v>
+        <v>640.42999999999995</v>
       </c>
       <c r="D32">
-        <v>426.76</v>
+        <v>695.7</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>3291.7</v>
+        <v>3818.9</v>
       </c>
       <c r="B33">
-        <v>261.58999999999997</v>
+        <v>554.32000000000005</v>
       </c>
       <c r="C33">
-        <v>276.94</v>
+        <v>660.58</v>
       </c>
       <c r="D33">
-        <v>437.35</v>
+        <v>711.3</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>3497.7</v>
+        <v>4024.2</v>
       </c>
       <c r="B34">
-        <v>271.89</v>
+        <v>576.51</v>
       </c>
       <c r="C34">
-        <v>284.95</v>
+        <v>678.63</v>
       </c>
       <c r="D34">
-        <v>446.95</v>
+        <v>722.76</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>3706.8</v>
+        <v>4229.5</v>
       </c>
       <c r="B35">
-        <v>281.55</v>
+        <v>597.13</v>
       </c>
       <c r="C35">
-        <v>292.20999999999998</v>
+        <v>694.45</v>
       </c>
       <c r="D35">
-        <v>455.65</v>
+        <v>730.54</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>3919</v>
+        <v>4434.8</v>
       </c>
       <c r="B36">
-        <v>290.58</v>
+        <v>616.12</v>
       </c>
       <c r="C36">
-        <v>298.8</v>
+        <v>707.87</v>
       </c>
       <c r="D36">
-        <v>463.56</v>
+        <v>737.42</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>4134.3</v>
+        <v>4662.5</v>
       </c>
       <c r="B37">
-        <v>299.04000000000002</v>
+        <v>635.20000000000005</v>
       </c>
       <c r="C37">
-        <v>304.79000000000002</v>
+        <v>719.77</v>
       </c>
       <c r="D37">
-        <v>470.77</v>
+        <v>751.99</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>4352.5</v>
+        <v>4903.8</v>
       </c>
       <c r="B38">
-        <v>306.95</v>
+        <v>653.52</v>
       </c>
       <c r="C38">
-        <v>310.24</v>
+        <v>729.24</v>
       </c>
       <c r="D38">
-        <v>477.36</v>
+        <v>770.55</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>4573.7</v>
+        <v>5137.5</v>
       </c>
       <c r="B39">
-        <v>314.35000000000002</v>
+        <v>669.77</v>
       </c>
       <c r="C39">
-        <v>315.20999999999998</v>
+        <v>738.8</v>
       </c>
       <c r="D39">
-        <v>483.4</v>
+        <v>788.61</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>4797.8999999999996</v>
+        <v>5371.1</v>
       </c>
       <c r="B40">
-        <v>321.27999999999997</v>
+        <v>685.18</v>
       </c>
       <c r="C40">
-        <v>319.76</v>
+        <v>757.62</v>
       </c>
       <c r="D40">
-        <v>488.98</v>
+        <v>806.66</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>5025.2</v>
+        <v>5550</v>
       </c>
       <c r="B41">
-        <v>327.79</v>
+        <v>696.16</v>
       </c>
       <c r="C41">
-        <v>323.93</v>
+        <v>772.38</v>
       </c>
       <c r="D41">
-        <v>494.13</v>
+        <v>819.59</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>5255.5</v>
+        <v>5728.9</v>
       </c>
       <c r="B42">
-        <v>333.9</v>
+        <v>706.42</v>
       </c>
       <c r="C42">
-        <v>327.76</v>
+        <v>786.77</v>
       </c>
       <c r="D42">
-        <v>498.93</v>
+        <v>831.75</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>5489</v>
+        <v>5907.8</v>
       </c>
       <c r="B43">
-        <v>339.65</v>
+        <v>715.87</v>
       </c>
       <c r="C43">
-        <v>331.29</v>
+        <v>800.41</v>
       </c>
       <c r="D43">
-        <v>503.41</v>
+        <v>843.16</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>5725.6</v>
+        <v>6086.7</v>
       </c>
       <c r="B44">
-        <v>345.06</v>
+        <v>723.88</v>
       </c>
       <c r="C44">
-        <v>334.57</v>
+        <v>813.08</v>
       </c>
       <c r="D44">
-        <v>507.61</v>
+        <v>853.83</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>5965.6</v>
+        <v>6265.6</v>
       </c>
       <c r="B45">
-        <v>350.18</v>
+        <v>729.75</v>
       </c>
       <c r="C45">
-        <v>337.61</v>
+        <v>824.52</v>
       </c>
       <c r="D45">
-        <v>511.56</v>
+        <v>863.74</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>6208.8</v>
+        <v>6444.5</v>
       </c>
       <c r="B46">
-        <v>355.02</v>
+        <v>734.9</v>
       </c>
       <c r="C46">
-        <v>340.44</v>
+        <v>834.71</v>
       </c>
       <c r="D46">
-        <v>515.29999999999995</v>
+        <v>872.87</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>6455.3</v>
+        <v>6623.4</v>
       </c>
       <c r="B47">
-        <v>359.61</v>
+        <v>746.1</v>
       </c>
       <c r="C47">
-        <v>343.1</v>
+        <v>844.1</v>
       </c>
       <c r="D47">
-        <v>518.85</v>
+        <v>881.38</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>6705.3</v>
+        <v>6816.1</v>
       </c>
       <c r="B48">
-        <v>363.97</v>
+        <v>762.29</v>
       </c>
       <c r="C48">
-        <v>345.58</v>
+        <v>853.81</v>
       </c>
       <c r="D48">
-        <v>522.22</v>
+        <v>889.99</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>6958.6</v>
+        <v>6999.9</v>
       </c>
       <c r="B49">
-        <v>368.12</v>
+        <v>777.98</v>
       </c>
       <c r="C49">
-        <v>347.92</v>
+        <v>863.47</v>
       </c>
       <c r="D49">
-        <v>525.44000000000005</v>
+        <v>898.09</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>7215.4</v>
+        <v>7165.8</v>
       </c>
       <c r="B50">
-        <v>372.08</v>
+        <v>791.69</v>
       </c>
       <c r="C50">
-        <v>350.13</v>
+        <v>872.55</v>
       </c>
       <c r="D50">
-        <v>528.53</v>
+        <v>905.45</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>7475.8</v>
+        <v>7331.8</v>
       </c>
       <c r="B51">
-        <v>375.85</v>
+        <v>804.65</v>
       </c>
       <c r="C51">
-        <v>352.22</v>
+        <v>881.51</v>
       </c>
       <c r="D51">
-        <v>531.49</v>
+        <v>912.72</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>7739.2</v>
+        <v>7497.8</v>
       </c>
       <c r="B52">
-        <v>379.46</v>
+        <v>816.82</v>
       </c>
       <c r="C52">
-        <v>354.2</v>
+        <v>890.23</v>
       </c>
       <c r="D52">
-        <v>534.34</v>
+        <v>919.86</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>8006.3</v>
+        <v>7663.7</v>
       </c>
       <c r="B53">
-        <v>382.93</v>
+        <v>828.25</v>
       </c>
       <c r="C53">
-        <v>356.08</v>
+        <v>898.66</v>
       </c>
       <c r="D53">
-        <v>537.09</v>
+        <v>926.85</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>8277.1</v>
+        <v>7829.7</v>
       </c>
       <c r="B54">
-        <v>386.25</v>
+        <v>838.99</v>
       </c>
       <c r="C54">
-        <v>357.87</v>
+        <v>906.75</v>
       </c>
       <c r="D54">
-        <v>539.74</v>
+        <v>933.67</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>8551.2000000000007</v>
+        <v>7995.6</v>
       </c>
       <c r="B55">
-        <v>389.44</v>
+        <v>849.1</v>
       </c>
       <c r="C55">
-        <v>359.59</v>
+        <v>914.51</v>
       </c>
       <c r="D55">
-        <v>542.30999999999995</v>
+        <v>940.29</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>8828.7999999999993</v>
+        <v>8161.6</v>
       </c>
       <c r="B56">
-        <v>392.51</v>
+        <v>858.65</v>
       </c>
       <c r="C56">
-        <v>361.22</v>
+        <v>921.95</v>
       </c>
       <c r="D56">
-        <v>544.79999999999995</v>
+        <v>946.7</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57">
+        <v>8327.5</v>
+      </c>
+      <c r="B57">
+        <v>867.69</v>
+      </c>
+      <c r="C57">
+        <v>929.07</v>
+      </c>
+      <c r="D57">
+        <v>952.91</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>8493.5</v>
+      </c>
+      <c r="B58">
+        <v>876.26</v>
+      </c>
+      <c r="C58">
+        <v>935.9</v>
+      </c>
+      <c r="D58">
+        <v>958.91</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>8659.4</v>
+      </c>
+      <c r="B59">
+        <v>884.41</v>
+      </c>
+      <c r="C59">
+        <v>942.45</v>
+      </c>
+      <c r="D59">
+        <v>964.7</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>8825.4</v>
+      </c>
+      <c r="B60">
+        <v>891.43</v>
+      </c>
+      <c r="C60">
+        <v>947.28</v>
+      </c>
+      <c r="D60">
+        <v>969.57</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61">
         <v>9000</v>
       </c>
-      <c r="B57">
-        <v>394.34</v>
-      </c>
-      <c r="C57">
-        <v>362.18</v>
-      </c>
-      <c r="D57">
-        <v>546.27</v>
+      <c r="B61">
+        <v>899.06</v>
+      </c>
+      <c r="C61">
+        <v>953.77</v>
+      </c>
+      <c r="D61">
+        <v>975.11</v>
       </c>
     </row>
   </sheetData>
@@ -1250,7 +1306,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3985F16-6493-457D-8950-27801BD1F8FD}">
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -1286,13 +1342,13 @@
         <v>90</v>
       </c>
       <c r="B3">
-        <v>20.059000000000001</v>
+        <v>20.073</v>
       </c>
       <c r="C3">
-        <v>20.004999999999999</v>
+        <v>20.024999999999999</v>
       </c>
       <c r="D3">
-        <v>20.152999999999999</v>
+        <v>20.225000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1300,783 +1356,699 @@
         <v>120</v>
       </c>
       <c r="B4">
-        <v>20.103999999999999</v>
+        <v>20.111999999999998</v>
       </c>
       <c r="C4">
-        <v>20.015000000000001</v>
+        <v>20.047000000000001</v>
       </c>
       <c r="D4">
-        <v>20.27</v>
+        <v>20.34</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>146.16999999999999</v>
+        <v>146.49</v>
       </c>
       <c r="B5">
-        <v>20.155999999999999</v>
+        <v>20.158999999999999</v>
       </c>
       <c r="C5">
-        <v>20.027999999999999</v>
+        <v>20.074000000000002</v>
       </c>
       <c r="D5">
-        <v>20.408999999999999</v>
+        <v>20.481999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>172.34</v>
+        <v>172.98</v>
       </c>
       <c r="B6">
-        <v>20.225999999999999</v>
+        <v>20.224</v>
       </c>
       <c r="C6">
-        <v>20.05</v>
+        <v>20.111000000000001</v>
       </c>
       <c r="D6">
-        <v>20.599</v>
+        <v>20.678000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>207.5</v>
+        <v>209.33</v>
       </c>
       <c r="B7">
-        <v>20.361999999999998</v>
+        <v>20.353000000000002</v>
       </c>
       <c r="C7">
-        <v>20.099</v>
+        <v>20.187999999999999</v>
       </c>
       <c r="D7">
-        <v>20.978999999999999</v>
+        <v>21.084</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>253.01</v>
+        <v>256.45</v>
       </c>
       <c r="B8">
-        <v>20.625</v>
+        <v>20.609000000000002</v>
       </c>
       <c r="C8">
-        <v>20.212</v>
+        <v>20.356999999999999</v>
       </c>
       <c r="D8">
-        <v>21.748000000000001</v>
+        <v>21.920999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>305.99</v>
+        <v>311.10000000000002</v>
       </c>
       <c r="B9">
-        <v>21.071999999999999</v>
+        <v>21.047999999999998</v>
       </c>
       <c r="C9">
-        <v>20.449000000000002</v>
+        <v>20.701000000000001</v>
       </c>
       <c r="D9">
-        <v>23.108000000000001</v>
+        <v>23.405999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>364.48</v>
+        <v>371.39</v>
       </c>
       <c r="B10">
-        <v>21.757000000000001</v>
+        <v>21.734999999999999</v>
       </c>
       <c r="C10">
-        <v>20.887</v>
+        <v>21.338999999999999</v>
       </c>
       <c r="D10">
-        <v>25.248999999999999</v>
+        <v>25.759</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>429.25</v>
+        <v>438.22</v>
       </c>
       <c r="B11">
-        <v>22.774000000000001</v>
+        <v>22.774999999999999</v>
       </c>
       <c r="C11">
-        <v>21.66</v>
+        <v>22.46</v>
       </c>
       <c r="D11">
-        <v>28.530999999999999</v>
+        <v>29.302</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>475.71</v>
+        <v>513.58000000000004</v>
       </c>
       <c r="B12">
-        <v>23.641999999999999</v>
+        <v>24.334</v>
       </c>
       <c r="C12">
-        <v>22.384</v>
+        <v>24.367999999999999</v>
       </c>
       <c r="D12">
-        <v>31.356999999999999</v>
+        <v>34.481999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>522.16</v>
+        <v>598.55999999999995</v>
       </c>
       <c r="B13">
-        <v>24.652000000000001</v>
+        <v>26.625</v>
       </c>
       <c r="C13">
-        <v>23.298999999999999</v>
+        <v>27.466000000000001</v>
       </c>
       <c r="D13">
-        <v>34.649000000000001</v>
+        <v>41.741999999999997</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>609.16</v>
+        <v>692.56</v>
       </c>
       <c r="B14">
-        <v>27.01</v>
+        <v>29.859000000000002</v>
       </c>
       <c r="C14">
-        <v>25.747</v>
+        <v>32.170999999999999</v>
       </c>
       <c r="D14">
-        <v>42.023000000000003</v>
+        <v>51.338000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>780.76</v>
+        <v>793.89</v>
       </c>
       <c r="B15">
-        <v>33.365000000000002</v>
+        <v>34.212000000000003</v>
       </c>
       <c r="C15">
-        <v>33.31</v>
+        <v>38.805999999999997</v>
       </c>
       <c r="D15">
-        <v>60.511000000000003</v>
+        <v>63.27</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>857.25</v>
+        <v>901.06</v>
       </c>
       <c r="B16">
-        <v>36.505000000000003</v>
+        <v>39.819000000000003</v>
       </c>
       <c r="C16">
-        <v>37.207999999999998</v>
+        <v>47.564999999999998</v>
       </c>
       <c r="D16">
-        <v>69.221000000000004</v>
+        <v>77.393000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>933.74</v>
+        <v>1013.7</v>
       </c>
       <c r="B17">
-        <v>39.942</v>
+        <v>46.819000000000003</v>
       </c>
       <c r="C17">
-        <v>41.536999999999999</v>
+        <v>58.563000000000002</v>
       </c>
       <c r="D17">
-        <v>78.512</v>
+        <v>93.585999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>1001.6</v>
+        <v>1132.5</v>
       </c>
       <c r="B18">
-        <v>43.204999999999998</v>
+        <v>55.375999999999998</v>
       </c>
       <c r="C18">
-        <v>45.707000000000001</v>
+        <v>71.894999999999996</v>
       </c>
       <c r="D18">
-        <v>87.022000000000006</v>
+        <v>111.83</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>1069.5</v>
+        <v>1259</v>
       </c>
       <c r="B19">
-        <v>46.661999999999999</v>
+        <v>65.676000000000002</v>
       </c>
       <c r="C19">
-        <v>50.167999999999999</v>
+        <v>87.649000000000001</v>
       </c>
       <c r="D19">
-        <v>95.71</v>
+        <v>132.15</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>1137.3</v>
+        <v>1394.7</v>
       </c>
       <c r="B20">
-        <v>50.293999999999997</v>
+        <v>79.13</v>
       </c>
       <c r="C20">
-        <v>54.878</v>
+        <v>109.16</v>
       </c>
       <c r="D20">
-        <v>104.5</v>
+        <v>156.54</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>1205.2</v>
+        <v>1466.9</v>
       </c>
       <c r="B21">
-        <v>54.084000000000003</v>
+        <v>86.676000000000002</v>
       </c>
       <c r="C21">
-        <v>59.798999999999999</v>
+        <v>120.84</v>
       </c>
       <c r="D21">
-        <v>113.34</v>
+        <v>169.76</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>1341.4</v>
+        <v>1539.1</v>
       </c>
       <c r="B22">
-        <v>62.182000000000002</v>
+        <v>94.554000000000002</v>
       </c>
       <c r="C22">
-        <v>70.234999999999999</v>
+        <v>132.69</v>
       </c>
       <c r="D22">
-        <v>130.91</v>
+        <v>183.14</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>1477.6</v>
+        <v>1702.8</v>
       </c>
       <c r="B23">
-        <v>70.635999999999996</v>
+        <v>113.56</v>
       </c>
       <c r="C23">
-        <v>80.977999999999994</v>
+        <v>159.91999999999999</v>
       </c>
       <c r="D23">
-        <v>148.06</v>
+        <v>213.55</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>1621.9</v>
+        <v>1866.5</v>
       </c>
       <c r="B24">
-        <v>79.852999999999994</v>
+        <v>133.35</v>
       </c>
       <c r="C24">
-        <v>92.465999999999994</v>
+        <v>187.26</v>
       </c>
       <c r="D24">
-        <v>165.59</v>
+        <v>243.6</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>1772</v>
+        <v>2063.6999999999998</v>
       </c>
       <c r="B25">
-        <v>89.590999999999994</v>
+        <v>157.77000000000001</v>
       </c>
       <c r="C25">
-        <v>104.34</v>
+        <v>219.69</v>
       </c>
       <c r="D25">
-        <v>183.03</v>
+        <v>278.7</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>1928.9</v>
+        <v>2276.1</v>
       </c>
       <c r="B26">
-        <v>99.802999999999997</v>
+        <v>184.26</v>
       </c>
       <c r="C26">
-        <v>116.48</v>
+        <v>253.64</v>
       </c>
       <c r="D26">
-        <v>200.29</v>
+        <v>314.87</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>2091.6</v>
+        <v>2500.8000000000002</v>
       </c>
       <c r="B27">
-        <v>110.32</v>
+        <v>212.14</v>
       </c>
       <c r="C27">
-        <v>128.66999999999999</v>
+        <v>288.13</v>
       </c>
       <c r="D27">
-        <v>217.14</v>
+        <v>351.05</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>2260.4</v>
+        <v>2735.5</v>
       </c>
       <c r="B28">
-        <v>121.07</v>
+        <v>240.81</v>
       </c>
       <c r="C28">
-        <v>140.79</v>
+        <v>322.45</v>
       </c>
       <c r="D28">
-        <v>233.5</v>
+        <v>386.52</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>2435.1</v>
+        <v>2977.2</v>
       </c>
       <c r="B29">
-        <v>131.93</v>
+        <v>269.69</v>
       </c>
       <c r="C29">
-        <v>152.71</v>
+        <v>355.94</v>
       </c>
       <c r="D29">
-        <v>249.26</v>
+        <v>420.61</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>2615.5</v>
+        <v>3223.1</v>
       </c>
       <c r="B30">
-        <v>142.79</v>
+        <v>298.26</v>
       </c>
       <c r="C30">
-        <v>164.3</v>
+        <v>388.1</v>
       </c>
       <c r="D30">
-        <v>264.33</v>
+        <v>452.86</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>2801.1</v>
+        <v>3470.7</v>
       </c>
       <c r="B31">
-        <v>153.56</v>
+        <v>326.16000000000003</v>
       </c>
       <c r="C31">
-        <v>175.48</v>
+        <v>418.64</v>
       </c>
       <c r="D31">
-        <v>278.62</v>
+        <v>483.03</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>2991.5</v>
+        <v>3718.4</v>
       </c>
       <c r="B32">
-        <v>164.14</v>
+        <v>353.15</v>
       </c>
       <c r="C32">
-        <v>186.16</v>
+        <v>447.44</v>
       </c>
       <c r="D32">
-        <v>292.10000000000002</v>
+        <v>511.07</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>3186.2</v>
+        <v>3966</v>
       </c>
       <c r="B33">
-        <v>174.45</v>
+        <v>379.21</v>
       </c>
       <c r="C33">
-        <v>196.28</v>
+        <v>474.59</v>
       </c>
       <c r="D33">
-        <v>304.72000000000003</v>
+        <v>537.16999999999996</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>3384.7</v>
+        <v>4213.6000000000004</v>
       </c>
       <c r="B34">
-        <v>184.44</v>
+        <v>404.35</v>
       </c>
       <c r="C34">
-        <v>205.81</v>
+        <v>500.2</v>
       </c>
       <c r="D34">
-        <v>316.49</v>
+        <v>561.47</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>3586.7</v>
+        <v>4461.3</v>
       </c>
       <c r="B35">
-        <v>194.05</v>
+        <v>428.57</v>
       </c>
       <c r="C35">
-        <v>214.74</v>
+        <v>524.37</v>
       </c>
       <c r="D35">
-        <v>327.42</v>
+        <v>584.16</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>3791.8</v>
+        <v>4708.8999999999996</v>
       </c>
       <c r="B36">
-        <v>203.27</v>
+        <v>451.88</v>
       </c>
       <c r="C36">
-        <v>223.07</v>
+        <v>547.21</v>
       </c>
       <c r="D36">
-        <v>337.53</v>
+        <v>605.37</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>3999.7</v>
+        <v>4956.5</v>
       </c>
       <c r="B37">
-        <v>212.06</v>
+        <v>474.3</v>
       </c>
       <c r="C37">
-        <v>230.81</v>
+        <v>568.79999999999995</v>
       </c>
       <c r="D37">
-        <v>346.86</v>
+        <v>625.16</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>4210.3</v>
+        <v>5204.2</v>
       </c>
       <c r="B38">
-        <v>220.43</v>
+        <v>495.85</v>
       </c>
       <c r="C38">
-        <v>237.99</v>
+        <v>589.21</v>
       </c>
       <c r="D38">
-        <v>355.46</v>
+        <v>643.62</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>4423.3</v>
+        <v>5451.8</v>
       </c>
       <c r="B39">
-        <v>228.38</v>
+        <v>516.53</v>
       </c>
       <c r="C39">
-        <v>244.63</v>
+        <v>608.48</v>
       </c>
       <c r="D39">
-        <v>363.38</v>
+        <v>660.79</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>4638.6000000000004</v>
+        <v>5699.4</v>
       </c>
       <c r="B40">
-        <v>235.92</v>
+        <v>536.37</v>
       </c>
       <c r="C40">
-        <v>250.78</v>
+        <v>626.63</v>
       </c>
       <c r="D40">
-        <v>370.67</v>
+        <v>676.71</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>4856.1000000000004</v>
+        <v>5947</v>
       </c>
       <c r="B41">
-        <v>243.06</v>
+        <v>555.36</v>
       </c>
       <c r="C41">
-        <v>256.45999999999998</v>
+        <v>643.69000000000005</v>
       </c>
       <c r="D41">
-        <v>377.39</v>
+        <v>691.34</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>5075.8999999999996</v>
+        <v>6194.7</v>
       </c>
       <c r="B42">
-        <v>249.82</v>
+        <v>573.5</v>
       </c>
       <c r="C42">
-        <v>261.70999999999998</v>
+        <v>659.64</v>
       </c>
       <c r="D42">
-        <v>383.59</v>
+        <v>704.52</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>5297.9</v>
+        <v>6442.3</v>
       </c>
       <c r="B43">
-        <v>256.20999999999998</v>
+        <v>590.75</v>
       </c>
       <c r="C43">
-        <v>266.58</v>
+        <v>674.43</v>
       </c>
       <c r="D43">
-        <v>389.31</v>
+        <v>715.9</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>5522.2</v>
+        <v>6689.9</v>
       </c>
       <c r="B44">
-        <v>262.27</v>
+        <v>607.04999999999995</v>
       </c>
       <c r="C44">
-        <v>271.08</v>
+        <v>687.89</v>
       </c>
       <c r="D44">
-        <v>394.61</v>
+        <v>724.88</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>5748.6</v>
+        <v>6939</v>
       </c>
       <c r="B45">
-        <v>268.01</v>
+        <v>622.33000000000004</v>
       </c>
       <c r="C45">
-        <v>275.26</v>
+        <v>699.8</v>
       </c>
       <c r="D45">
-        <v>399.52</v>
+        <v>730.85</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>5977.4</v>
+        <v>7188.1</v>
       </c>
       <c r="B46">
-        <v>273.44</v>
+        <v>636.47</v>
       </c>
       <c r="C46">
-        <v>279.14</v>
+        <v>710.13</v>
       </c>
       <c r="D46">
-        <v>404.08</v>
+        <v>736.33</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>6208.4</v>
+        <v>7462.2</v>
       </c>
       <c r="B47">
-        <v>278.60000000000002</v>
+        <v>650.66999999999996</v>
       </c>
       <c r="C47">
-        <v>282.76</v>
+        <v>719.66</v>
       </c>
       <c r="D47">
-        <v>408.33</v>
+        <v>746.51</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>6441.9</v>
+        <v>7756.4</v>
       </c>
       <c r="B48">
-        <v>283.49</v>
+        <v>664.58</v>
       </c>
       <c r="C48">
-        <v>286.13</v>
+        <v>727.93</v>
       </c>
       <c r="D48">
-        <v>412.3</v>
+        <v>760.59</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>6677.7</v>
+        <v>8047</v>
       </c>
       <c r="B49">
-        <v>288.14999999999998</v>
+        <v>677.29</v>
       </c>
       <c r="C49">
-        <v>289.27999999999997</v>
+        <v>734.96</v>
       </c>
       <c r="D49">
-        <v>416.02</v>
+        <v>775.1</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>6916</v>
+        <v>8318</v>
       </c>
       <c r="B50">
-        <v>292.57</v>
+        <v>688.43</v>
       </c>
       <c r="C50">
-        <v>292.23</v>
+        <v>745.78</v>
       </c>
       <c r="D50">
-        <v>419.52</v>
+        <v>788.5</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>7156.8</v>
+        <v>8564.7000000000007</v>
       </c>
       <c r="B51">
-        <v>296.79000000000002</v>
+        <v>698.11</v>
       </c>
       <c r="C51">
-        <v>294.99</v>
+        <v>758.4</v>
       </c>
       <c r="D51">
-        <v>422.81</v>
+        <v>800.44</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>7400.1</v>
+        <v>8811.5</v>
       </c>
       <c r="B52">
-        <v>300.81</v>
+        <v>707.3</v>
       </c>
       <c r="C52">
-        <v>297.58999999999997</v>
+        <v>771.31</v>
       </c>
       <c r="D52">
-        <v>425.91</v>
+        <v>811.9</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>7646</v>
+        <v>9000</v>
       </c>
       <c r="B53">
-        <v>304.64999999999998</v>
+        <v>713.69</v>
       </c>
       <c r="C53">
-        <v>300.05</v>
+        <v>779.9</v>
       </c>
       <c r="D53">
-        <v>428.86</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54">
-        <v>7894.4</v>
-      </c>
-      <c r="B54">
-        <v>308.32</v>
-      </c>
-      <c r="C54">
-        <v>302.36</v>
-      </c>
-      <c r="D54">
-        <v>431.65</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55">
-        <v>8145.5</v>
-      </c>
-      <c r="B55">
-        <v>311.83999999999997</v>
-      </c>
-      <c r="C55">
-        <v>304.55</v>
-      </c>
-      <c r="D55">
-        <v>434.31</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56">
-        <v>8399.1</v>
-      </c>
-      <c r="B56">
-        <v>315.20999999999998</v>
-      </c>
-      <c r="C56">
-        <v>306.63</v>
-      </c>
-      <c r="D56">
-        <v>436.85</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57">
-        <v>8655.4</v>
-      </c>
-      <c r="B57">
-        <v>318.44</v>
-      </c>
-      <c r="C57">
-        <v>308.61</v>
-      </c>
-      <c r="D57">
-        <v>439.27</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58">
-        <v>8914.2000000000007</v>
-      </c>
-      <c r="B58">
-        <v>321.55</v>
-      </c>
-      <c r="C58">
-        <v>310.49</v>
-      </c>
-      <c r="D58">
-        <v>441.6</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59">
-        <v>9000</v>
-      </c>
-      <c r="B59">
-        <v>322.56</v>
-      </c>
-      <c r="C59">
-        <v>311.10000000000002</v>
-      </c>
-      <c r="D59">
-        <v>442.35</v>
+        <v>819.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 4-side heating (Yakovlev) OGZ curves with visibility toggle
New Excel sheets carry temperatures for 1/2-layer GKL protection under
4-sided heating; wire them into the OGZ comparison chart alongside the
existing 3-sided variants, and let the user pick which curves to show
via a multiselect (also filters the Excel export).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/температура с ОГЗ.xlsx
+++ b/температура с ОГЗ.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YandexDisk\02_PROJECT\Python\steel\Steel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71609E93-A3D3-494A-B5FD-19737B461C96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3751B4C0-0200-421D-8845-8597BA7C6337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CF9B73C0-209F-4FC5-92E1-844AEABB6AA9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{CF9B73C0-209F-4FC5-92E1-844AEABB6AA9}"/>
   </bookViews>
   <sheets>
     <sheet name="1 слой ГКЛ" sheetId="1" r:id="rId1"/>
     <sheet name="2 слой ГКЛ" sheetId="2" r:id="rId2"/>
+    <sheet name="1 слой ГКЛ (методика Яковлева)" sheetId="3" r:id="rId3"/>
+    <sheet name="2 слоя ГКЛ (методика Яковлева)" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="4">
   <si>
     <t>time,s</t>
   </si>
@@ -2054,4 +2056,2614 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46B00F1-4333-4DDD-BE10-8E7DA9E6AE21}">
+  <dimension ref="A1:D105"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>90</v>
+      </c>
+      <c r="B3">
+        <v>23.855</v>
+      </c>
+      <c r="C3">
+        <v>21.094000000000001</v>
+      </c>
+      <c r="D3">
+        <v>23.855</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>120</v>
+      </c>
+      <c r="B4">
+        <v>25.734999999999999</v>
+      </c>
+      <c r="C4">
+        <v>21.651</v>
+      </c>
+      <c r="D4">
+        <v>25.734999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>145.81</v>
+      </c>
+      <c r="B5">
+        <v>27.869</v>
+      </c>
+      <c r="C5">
+        <v>22.324000000000002</v>
+      </c>
+      <c r="D5">
+        <v>27.869</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>171.61</v>
+      </c>
+      <c r="B6">
+        <v>30.56</v>
+      </c>
+      <c r="C6">
+        <v>23.248999999999999</v>
+      </c>
+      <c r="D6">
+        <v>30.56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>207.98</v>
+      </c>
+      <c r="B7">
+        <v>35.448999999999998</v>
+      </c>
+      <c r="C7">
+        <v>25.204999999999998</v>
+      </c>
+      <c r="D7">
+        <v>35.448999999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>248.94</v>
+      </c>
+      <c r="B8">
+        <v>42.247999999999998</v>
+      </c>
+      <c r="C8">
+        <v>28.428999999999998</v>
+      </c>
+      <c r="D8">
+        <v>42.247999999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>294.39</v>
+      </c>
+      <c r="B9">
+        <v>51.192</v>
+      </c>
+      <c r="C9">
+        <v>33.44</v>
+      </c>
+      <c r="D9">
+        <v>51.191000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>343.97</v>
+      </c>
+      <c r="B10">
+        <v>62.359000000000002</v>
+      </c>
+      <c r="C10">
+        <v>40.704999999999998</v>
+      </c>
+      <c r="D10">
+        <v>62.357999999999997</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>397.48</v>
+      </c>
+      <c r="B11">
+        <v>75.754000000000005</v>
+      </c>
+      <c r="C11">
+        <v>50.582999999999998</v>
+      </c>
+      <c r="D11">
+        <v>75.754000000000005</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>455.2</v>
+      </c>
+      <c r="B12">
+        <v>91.445999999999998</v>
+      </c>
+      <c r="C12">
+        <v>63.375999999999998</v>
+      </c>
+      <c r="D12">
+        <v>91.445999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>518.21</v>
+      </c>
+      <c r="B13">
+        <v>109.7</v>
+      </c>
+      <c r="C13">
+        <v>79.454999999999998</v>
+      </c>
+      <c r="D13">
+        <v>109.7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>588.52</v>
+      </c>
+      <c r="B14">
+        <v>131.04</v>
+      </c>
+      <c r="C14">
+        <v>99.382999999999996</v>
+      </c>
+      <c r="D14">
+        <v>131.04</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>669.01</v>
+      </c>
+      <c r="B15">
+        <v>156.26</v>
+      </c>
+      <c r="C15">
+        <v>123.92</v>
+      </c>
+      <c r="D15">
+        <v>156.26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>763</v>
+      </c>
+      <c r="B16">
+        <v>186.2</v>
+      </c>
+      <c r="C16">
+        <v>153.9</v>
+      </c>
+      <c r="D16">
+        <v>186.19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>873.8</v>
+      </c>
+      <c r="B17">
+        <v>221.47</v>
+      </c>
+      <c r="C17">
+        <v>189.87</v>
+      </c>
+      <c r="D17">
+        <v>221.47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>1002.7</v>
+      </c>
+      <c r="B18">
+        <v>261.8</v>
+      </c>
+      <c r="C18">
+        <v>231.45</v>
+      </c>
+      <c r="D18">
+        <v>261.8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>1148.2</v>
+      </c>
+      <c r="B19">
+        <v>305.75</v>
+      </c>
+      <c r="C19">
+        <v>277.02999999999997</v>
+      </c>
+      <c r="D19">
+        <v>305.75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>1305.5999999999999</v>
+      </c>
+      <c r="B20">
+        <v>351.06</v>
+      </c>
+      <c r="C20">
+        <v>324.19</v>
+      </c>
+      <c r="D20">
+        <v>351.06</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>1468.8</v>
+      </c>
+      <c r="B21">
+        <v>395.38</v>
+      </c>
+      <c r="C21">
+        <v>370.41</v>
+      </c>
+      <c r="D21">
+        <v>395.38</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>1632</v>
+      </c>
+      <c r="B22">
+        <v>437.01</v>
+      </c>
+      <c r="C22">
+        <v>413.9</v>
+      </c>
+      <c r="D22">
+        <v>437.01</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>1795.2</v>
+      </c>
+      <c r="B23">
+        <v>476.4</v>
+      </c>
+      <c r="C23">
+        <v>455.6</v>
+      </c>
+      <c r="D23">
+        <v>476.4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>1958.4</v>
+      </c>
+      <c r="B24">
+        <v>513.27</v>
+      </c>
+      <c r="C24">
+        <v>494.51</v>
+      </c>
+      <c r="D24">
+        <v>513.27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>2121.6</v>
+      </c>
+      <c r="B25">
+        <v>547.69000000000005</v>
+      </c>
+      <c r="C25">
+        <v>530.72</v>
+      </c>
+      <c r="D25">
+        <v>547.69000000000005</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>2284.8000000000002</v>
+      </c>
+      <c r="B26">
+        <v>579.79</v>
+      </c>
+      <c r="C26">
+        <v>564.4</v>
+      </c>
+      <c r="D26">
+        <v>579.79</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>2448.1</v>
+      </c>
+      <c r="B27">
+        <v>609.66</v>
+      </c>
+      <c r="C27">
+        <v>595.71</v>
+      </c>
+      <c r="D27">
+        <v>609.66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>2611.3000000000002</v>
+      </c>
+      <c r="B28">
+        <v>637.16999999999996</v>
+      </c>
+      <c r="C28">
+        <v>624.6</v>
+      </c>
+      <c r="D28">
+        <v>637.16999999999996</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>2774.5</v>
+      </c>
+      <c r="B29">
+        <v>662.19</v>
+      </c>
+      <c r="C29">
+        <v>650.95000000000005</v>
+      </c>
+      <c r="D29">
+        <v>662.19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>2937.7</v>
+      </c>
+      <c r="B30">
+        <v>684.46</v>
+      </c>
+      <c r="C30">
+        <v>674.53</v>
+      </c>
+      <c r="D30">
+        <v>684.46</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>3100.9</v>
+      </c>
+      <c r="B31">
+        <v>703.43</v>
+      </c>
+      <c r="C31">
+        <v>694.95</v>
+      </c>
+      <c r="D31">
+        <v>703.43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>3264.1</v>
+      </c>
+      <c r="B32">
+        <v>717.89</v>
+      </c>
+      <c r="C32">
+        <v>711.19</v>
+      </c>
+      <c r="D32">
+        <v>717.89</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>3427.3</v>
+      </c>
+      <c r="B33">
+        <v>727.53</v>
+      </c>
+      <c r="C33">
+        <v>722.86</v>
+      </c>
+      <c r="D33">
+        <v>727.53</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>3508.9</v>
+      </c>
+      <c r="B34">
+        <v>730.95</v>
+      </c>
+      <c r="C34">
+        <v>727.71</v>
+      </c>
+      <c r="D34">
+        <v>730.95</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>3590.5</v>
+      </c>
+      <c r="B35">
+        <v>733.59</v>
+      </c>
+      <c r="C35">
+        <v>730.9</v>
+      </c>
+      <c r="D35">
+        <v>733.59</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>3709.5</v>
+      </c>
+      <c r="B36">
+        <v>738.77</v>
+      </c>
+      <c r="C36">
+        <v>734.13</v>
+      </c>
+      <c r="D36">
+        <v>738.77</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>3834.1</v>
+      </c>
+      <c r="B37">
+        <v>747.69</v>
+      </c>
+      <c r="C37">
+        <v>738.83</v>
+      </c>
+      <c r="D37">
+        <v>747.69</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>3958.8</v>
+      </c>
+      <c r="B38">
+        <v>759.29</v>
+      </c>
+      <c r="C38">
+        <v>747.15</v>
+      </c>
+      <c r="D38">
+        <v>759.29</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>4095.6</v>
+      </c>
+      <c r="B39">
+        <v>773.7</v>
+      </c>
+      <c r="C39">
+        <v>760.91</v>
+      </c>
+      <c r="D39">
+        <v>773.7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>4206.3</v>
+      </c>
+      <c r="B40">
+        <v>786.05</v>
+      </c>
+      <c r="C40">
+        <v>773.91</v>
+      </c>
+      <c r="D40">
+        <v>786.05</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>4299.5</v>
+      </c>
+      <c r="B41">
+        <v>796.77</v>
+      </c>
+      <c r="C41">
+        <v>785.67</v>
+      </c>
+      <c r="D41">
+        <v>796.77</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>4392.7</v>
+      </c>
+      <c r="B42">
+        <v>807.58</v>
+      </c>
+      <c r="C42">
+        <v>797.55</v>
+      </c>
+      <c r="D42">
+        <v>807.58</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>4471.8</v>
+      </c>
+      <c r="B43">
+        <v>816.78</v>
+      </c>
+      <c r="C43">
+        <v>807.73</v>
+      </c>
+      <c r="D43">
+        <v>816.78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>4545.3</v>
+      </c>
+      <c r="B44">
+        <v>825.28</v>
+      </c>
+      <c r="C44">
+        <v>817.1</v>
+      </c>
+      <c r="D44">
+        <v>825.28</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>4618.7</v>
+      </c>
+      <c r="B45">
+        <v>833.66</v>
+      </c>
+      <c r="C45">
+        <v>826.22</v>
+      </c>
+      <c r="D45">
+        <v>833.66</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>4692.2</v>
+      </c>
+      <c r="B46">
+        <v>841.88</v>
+      </c>
+      <c r="C46">
+        <v>835.08</v>
+      </c>
+      <c r="D46">
+        <v>841.88</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>4765.7</v>
+      </c>
+      <c r="B47">
+        <v>849.91</v>
+      </c>
+      <c r="C47">
+        <v>843.65</v>
+      </c>
+      <c r="D47">
+        <v>849.91</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>4839.2</v>
+      </c>
+      <c r="B48">
+        <v>857.72</v>
+      </c>
+      <c r="C48">
+        <v>851.93</v>
+      </c>
+      <c r="D48">
+        <v>857.72</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>4912.7</v>
+      </c>
+      <c r="B49">
+        <v>865.32</v>
+      </c>
+      <c r="C49">
+        <v>859.93</v>
+      </c>
+      <c r="D49">
+        <v>865.32</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>4986.2</v>
+      </c>
+      <c r="B50">
+        <v>872.69</v>
+      </c>
+      <c r="C50">
+        <v>867.63</v>
+      </c>
+      <c r="D50">
+        <v>872.69</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>5059.7</v>
+      </c>
+      <c r="B51">
+        <v>879.82</v>
+      </c>
+      <c r="C51">
+        <v>875.07</v>
+      </c>
+      <c r="D51">
+        <v>879.82</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>5133.2</v>
+      </c>
+      <c r="B52">
+        <v>886.71</v>
+      </c>
+      <c r="C52">
+        <v>882.23</v>
+      </c>
+      <c r="D52">
+        <v>886.71</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>5206.7</v>
+      </c>
+      <c r="B53">
+        <v>893.37</v>
+      </c>
+      <c r="C53">
+        <v>889.13</v>
+      </c>
+      <c r="D53">
+        <v>893.37</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>5280.2</v>
+      </c>
+      <c r="B54">
+        <v>899.8</v>
+      </c>
+      <c r="C54">
+        <v>895.78</v>
+      </c>
+      <c r="D54">
+        <v>899.8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>5353.7</v>
+      </c>
+      <c r="B55">
+        <v>905.98</v>
+      </c>
+      <c r="C55">
+        <v>902.17</v>
+      </c>
+      <c r="D55">
+        <v>905.98</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>5427.2</v>
+      </c>
+      <c r="B56">
+        <v>911.57</v>
+      </c>
+      <c r="C56">
+        <v>907.42</v>
+      </c>
+      <c r="D56">
+        <v>911.57</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>5500.7</v>
+      </c>
+      <c r="B57">
+        <v>916.88</v>
+      </c>
+      <c r="C57">
+        <v>912.52</v>
+      </c>
+      <c r="D57">
+        <v>916.88</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>5574.2</v>
+      </c>
+      <c r="B58">
+        <v>921.96</v>
+      </c>
+      <c r="C58">
+        <v>917.5</v>
+      </c>
+      <c r="D58">
+        <v>921.96</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>5647.7</v>
+      </c>
+      <c r="B59">
+        <v>926.84</v>
+      </c>
+      <c r="C59">
+        <v>922.36</v>
+      </c>
+      <c r="D59">
+        <v>926.84</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>5721.2</v>
+      </c>
+      <c r="B60">
+        <v>931.54</v>
+      </c>
+      <c r="C60">
+        <v>927.1</v>
+      </c>
+      <c r="D60">
+        <v>931.54</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>5794.7</v>
+      </c>
+      <c r="B61">
+        <v>936.07</v>
+      </c>
+      <c r="C61">
+        <v>931.71</v>
+      </c>
+      <c r="D61">
+        <v>936.07</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>5868.2</v>
+      </c>
+      <c r="B62">
+        <v>940.46</v>
+      </c>
+      <c r="C62">
+        <v>936.19</v>
+      </c>
+      <c r="D62">
+        <v>940.46</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>5941.7</v>
+      </c>
+      <c r="B63">
+        <v>944.7</v>
+      </c>
+      <c r="C63">
+        <v>940.53</v>
+      </c>
+      <c r="D63">
+        <v>944.7</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>6015.2</v>
+      </c>
+      <c r="B64">
+        <v>948.8</v>
+      </c>
+      <c r="C64">
+        <v>944.75</v>
+      </c>
+      <c r="D64">
+        <v>948.8</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>6088.7</v>
+      </c>
+      <c r="B65">
+        <v>952.78</v>
+      </c>
+      <c r="C65">
+        <v>948.84</v>
+      </c>
+      <c r="D65">
+        <v>952.78</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>6162.2</v>
+      </c>
+      <c r="B66">
+        <v>956.64</v>
+      </c>
+      <c r="C66">
+        <v>952.82</v>
+      </c>
+      <c r="D66">
+        <v>956.64</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>6235.7</v>
+      </c>
+      <c r="B67">
+        <v>960.39</v>
+      </c>
+      <c r="C67">
+        <v>956.67</v>
+      </c>
+      <c r="D67">
+        <v>960.39</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>6309.2</v>
+      </c>
+      <c r="B68">
+        <v>964.03</v>
+      </c>
+      <c r="C68">
+        <v>960.41</v>
+      </c>
+      <c r="D68">
+        <v>964.03</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>6382.6</v>
+      </c>
+      <c r="B69">
+        <v>967.56</v>
+      </c>
+      <c r="C69">
+        <v>964.05</v>
+      </c>
+      <c r="D69">
+        <v>967.56</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>6456.1</v>
+      </c>
+      <c r="B70">
+        <v>970.99</v>
+      </c>
+      <c r="C70">
+        <v>967.58</v>
+      </c>
+      <c r="D70">
+        <v>970.99</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>6529.6</v>
+      </c>
+      <c r="B71">
+        <v>974.34</v>
+      </c>
+      <c r="C71">
+        <v>971.02</v>
+      </c>
+      <c r="D71">
+        <v>974.34</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>6603.1</v>
+      </c>
+      <c r="B72">
+        <v>977.59</v>
+      </c>
+      <c r="C72">
+        <v>974.36</v>
+      </c>
+      <c r="D72">
+        <v>977.59</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>6676.6</v>
+      </c>
+      <c r="B73">
+        <v>980.75</v>
+      </c>
+      <c r="C73">
+        <v>977.61</v>
+      </c>
+      <c r="D73">
+        <v>980.75</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>6750.1</v>
+      </c>
+      <c r="B74">
+        <v>983.83</v>
+      </c>
+      <c r="C74">
+        <v>980.77</v>
+      </c>
+      <c r="D74">
+        <v>983.83</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>6823.6</v>
+      </c>
+      <c r="B75">
+        <v>986.83</v>
+      </c>
+      <c r="C75">
+        <v>983.85</v>
+      </c>
+      <c r="D75">
+        <v>986.83</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>6897.1</v>
+      </c>
+      <c r="B76">
+        <v>989.76</v>
+      </c>
+      <c r="C76">
+        <v>986.86</v>
+      </c>
+      <c r="D76">
+        <v>989.76</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>6970.6</v>
+      </c>
+      <c r="B77">
+        <v>992.61</v>
+      </c>
+      <c r="C77">
+        <v>989.78</v>
+      </c>
+      <c r="D77">
+        <v>992.61</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>7044.1</v>
+      </c>
+      <c r="B78">
+        <v>995.4</v>
+      </c>
+      <c r="C78">
+        <v>992.64</v>
+      </c>
+      <c r="D78">
+        <v>995.4</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>7117.6</v>
+      </c>
+      <c r="B79">
+        <v>998.11</v>
+      </c>
+      <c r="C79">
+        <v>995.42</v>
+      </c>
+      <c r="D79">
+        <v>998.11</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>7191.1</v>
+      </c>
+      <c r="B80">
+        <v>1000.8</v>
+      </c>
+      <c r="C80">
+        <v>998.14</v>
+      </c>
+      <c r="D80">
+        <v>1000.8</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>7264.6</v>
+      </c>
+      <c r="B81">
+        <v>1003.4</v>
+      </c>
+      <c r="C81">
+        <v>1000.8</v>
+      </c>
+      <c r="D81">
+        <v>1003.4</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>7338.1</v>
+      </c>
+      <c r="B82">
+        <v>1005.9</v>
+      </c>
+      <c r="C82">
+        <v>1003.4</v>
+      </c>
+      <c r="D82">
+        <v>1005.9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>7411.6</v>
+      </c>
+      <c r="B83">
+        <v>1008.4</v>
+      </c>
+      <c r="C83">
+        <v>1005.9</v>
+      </c>
+      <c r="D83">
+        <v>1008.4</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>7485.1</v>
+      </c>
+      <c r="B84">
+        <v>1010.8</v>
+      </c>
+      <c r="C84">
+        <v>1008.4</v>
+      </c>
+      <c r="D84">
+        <v>1010.8</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>7558.6</v>
+      </c>
+      <c r="B85">
+        <v>1013.2</v>
+      </c>
+      <c r="C85">
+        <v>1010.8</v>
+      </c>
+      <c r="D85">
+        <v>1013.2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>7632.1</v>
+      </c>
+      <c r="B86">
+        <v>1015.5</v>
+      </c>
+      <c r="C86">
+        <v>1013.2</v>
+      </c>
+      <c r="D86">
+        <v>1015.5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>7705.6</v>
+      </c>
+      <c r="B87">
+        <v>1017.8</v>
+      </c>
+      <c r="C87">
+        <v>1015.5</v>
+      </c>
+      <c r="D87">
+        <v>1017.8</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>7779.1</v>
+      </c>
+      <c r="B88">
+        <v>1020</v>
+      </c>
+      <c r="C88">
+        <v>1017.8</v>
+      </c>
+      <c r="D88">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>7852.6</v>
+      </c>
+      <c r="B89">
+        <v>1022.2</v>
+      </c>
+      <c r="C89">
+        <v>1020</v>
+      </c>
+      <c r="D89">
+        <v>1022.2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>7926.1</v>
+      </c>
+      <c r="B90">
+        <v>1024.3</v>
+      </c>
+      <c r="C90">
+        <v>1022.2</v>
+      </c>
+      <c r="D90">
+        <v>1024.3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>7999.6</v>
+      </c>
+      <c r="B91">
+        <v>1026.4000000000001</v>
+      </c>
+      <c r="C91">
+        <v>1024.3</v>
+      </c>
+      <c r="D91">
+        <v>1026.4000000000001</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>8073.1</v>
+      </c>
+      <c r="B92">
+        <v>1028.5</v>
+      </c>
+      <c r="C92">
+        <v>1026.4000000000001</v>
+      </c>
+      <c r="D92">
+        <v>1028.5</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>8146.5</v>
+      </c>
+      <c r="B93">
+        <v>1030.5</v>
+      </c>
+      <c r="C93">
+        <v>1028.5</v>
+      </c>
+      <c r="D93">
+        <v>1030.5</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>8220</v>
+      </c>
+      <c r="B94">
+        <v>1032.5</v>
+      </c>
+      <c r="C94">
+        <v>1030.5</v>
+      </c>
+      <c r="D94">
+        <v>1032.5</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>8293.5</v>
+      </c>
+      <c r="B95">
+        <v>1034.5</v>
+      </c>
+      <c r="C95">
+        <v>1032.5</v>
+      </c>
+      <c r="D95">
+        <v>1034.5</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>8367</v>
+      </c>
+      <c r="B96">
+        <v>1036.4000000000001</v>
+      </c>
+      <c r="C96">
+        <v>1034.5</v>
+      </c>
+      <c r="D96">
+        <v>1036.4000000000001</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>8440.5</v>
+      </c>
+      <c r="B97">
+        <v>1038.3</v>
+      </c>
+      <c r="C97">
+        <v>1036.4000000000001</v>
+      </c>
+      <c r="D97">
+        <v>1038.3</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>8514</v>
+      </c>
+      <c r="B98">
+        <v>1040.0999999999999</v>
+      </c>
+      <c r="C98">
+        <v>1038.3</v>
+      </c>
+      <c r="D98">
+        <v>1040.0999999999999</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>8587.5</v>
+      </c>
+      <c r="B99">
+        <v>1041.9000000000001</v>
+      </c>
+      <c r="C99">
+        <v>1040.0999999999999</v>
+      </c>
+      <c r="D99">
+        <v>1041.9000000000001</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>8661</v>
+      </c>
+      <c r="B100">
+        <v>1043.7</v>
+      </c>
+      <c r="C100">
+        <v>1042</v>
+      </c>
+      <c r="D100">
+        <v>1043.7</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>8734.5</v>
+      </c>
+      <c r="B101">
+        <v>1045.5</v>
+      </c>
+      <c r="C101">
+        <v>1043.8</v>
+      </c>
+      <c r="D101">
+        <v>1045.5</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>8808</v>
+      </c>
+      <c r="B102">
+        <v>1047.2</v>
+      </c>
+      <c r="C102">
+        <v>1045.5</v>
+      </c>
+      <c r="D102">
+        <v>1047.2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>8881.5</v>
+      </c>
+      <c r="B103">
+        <v>1049</v>
+      </c>
+      <c r="C103">
+        <v>1047.3</v>
+      </c>
+      <c r="D103">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>8955</v>
+      </c>
+      <c r="B104">
+        <v>1050.5999999999999</v>
+      </c>
+      <c r="C104">
+        <v>1049</v>
+      </c>
+      <c r="D104">
+        <v>1050.5999999999999</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>9000</v>
+      </c>
+      <c r="B105">
+        <v>1051.5999999999999</v>
+      </c>
+      <c r="C105">
+        <v>1050</v>
+      </c>
+      <c r="D105">
+        <v>1051.5999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0C53F38-6AC1-4CBB-86E9-AF1803BAEABB}">
+  <dimension ref="A1:D80"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>90</v>
+      </c>
+      <c r="B3">
+        <v>20.268999999999998</v>
+      </c>
+      <c r="C3">
+        <v>20.073</v>
+      </c>
+      <c r="D3">
+        <v>20.268999999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>120</v>
+      </c>
+      <c r="B4">
+        <v>20.402999999999999</v>
+      </c>
+      <c r="C4">
+        <v>20.11</v>
+      </c>
+      <c r="D4">
+        <v>20.402999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>145.78</v>
+      </c>
+      <c r="B5">
+        <v>20.564</v>
+      </c>
+      <c r="C5">
+        <v>20.155000000000001</v>
+      </c>
+      <c r="D5">
+        <v>20.564</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>171.56</v>
+      </c>
+      <c r="B6">
+        <v>20.783999999999999</v>
+      </c>
+      <c r="C6">
+        <v>20.216000000000001</v>
+      </c>
+      <c r="D6">
+        <v>20.783999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>208.31</v>
+      </c>
+      <c r="B7">
+        <v>21.268000000000001</v>
+      </c>
+      <c r="C7">
+        <v>20.359000000000002</v>
+      </c>
+      <c r="D7">
+        <v>21.268000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>250.51</v>
+      </c>
+      <c r="B8">
+        <v>22.117000000000001</v>
+      </c>
+      <c r="C8">
+        <v>20.632000000000001</v>
+      </c>
+      <c r="D8">
+        <v>22.117000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>298.88</v>
+      </c>
+      <c r="B9">
+        <v>23.565000000000001</v>
+      </c>
+      <c r="C9">
+        <v>21.157</v>
+      </c>
+      <c r="D9">
+        <v>23.565000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>354.05</v>
+      </c>
+      <c r="B10">
+        <v>25.928000000000001</v>
+      </c>
+      <c r="C10">
+        <v>22.141999999999999</v>
+      </c>
+      <c r="D10">
+        <v>25.928000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>416.64</v>
+      </c>
+      <c r="B11">
+        <v>29.594999999999999</v>
+      </c>
+      <c r="C11">
+        <v>23.911000000000001</v>
+      </c>
+      <c r="D11">
+        <v>29.594999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>487.12</v>
+      </c>
+      <c r="B12">
+        <v>34.997999999999998</v>
+      </c>
+      <c r="C12">
+        <v>26.916</v>
+      </c>
+      <c r="D12">
+        <v>34.997999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>565.72</v>
+      </c>
+      <c r="B13">
+        <v>42.558</v>
+      </c>
+      <c r="C13">
+        <v>31.718</v>
+      </c>
+      <c r="D13">
+        <v>42.558</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>652.36</v>
+      </c>
+      <c r="B14">
+        <v>52.621000000000002</v>
+      </c>
+      <c r="C14">
+        <v>38.904000000000003</v>
+      </c>
+      <c r="D14">
+        <v>52.621000000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>746.69</v>
+      </c>
+      <c r="B15">
+        <v>65.37</v>
+      </c>
+      <c r="C15">
+        <v>48.923999999999999</v>
+      </c>
+      <c r="D15">
+        <v>65.37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>850.18</v>
+      </c>
+      <c r="B16">
+        <v>81.206999999999994</v>
+      </c>
+      <c r="C16">
+        <v>62.42</v>
+      </c>
+      <c r="D16">
+        <v>81.206999999999994</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>958.77</v>
+      </c>
+      <c r="B17">
+        <v>99.498999999999995</v>
+      </c>
+      <c r="C17">
+        <v>78.983999999999995</v>
+      </c>
+      <c r="D17">
+        <v>99.498999999999995</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>1075.0999999999999</v>
+      </c>
+      <c r="B18">
+        <v>120.57</v>
+      </c>
+      <c r="C18">
+        <v>98.933999999999997</v>
+      </c>
+      <c r="D18">
+        <v>120.57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>1200.4000000000001</v>
+      </c>
+      <c r="B19">
+        <v>144.52000000000001</v>
+      </c>
+      <c r="C19">
+        <v>122.34</v>
+      </c>
+      <c r="D19">
+        <v>144.52000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>1336.4</v>
+      </c>
+      <c r="B20">
+        <v>171.38</v>
+      </c>
+      <c r="C20">
+        <v>149.15</v>
+      </c>
+      <c r="D20">
+        <v>171.38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>1484.3</v>
+      </c>
+      <c r="B21">
+        <v>201.08</v>
+      </c>
+      <c r="C21">
+        <v>179.19</v>
+      </c>
+      <c r="D21">
+        <v>201.08</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>1644.6</v>
+      </c>
+      <c r="B22">
+        <v>233.29</v>
+      </c>
+      <c r="C22">
+        <v>212</v>
+      </c>
+      <c r="D22">
+        <v>233.29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>1816.6</v>
+      </c>
+      <c r="B23">
+        <v>267.33999999999997</v>
+      </c>
+      <c r="C23">
+        <v>246.78</v>
+      </c>
+      <c r="D23">
+        <v>267.33999999999997</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>1998.1</v>
+      </c>
+      <c r="B24">
+        <v>303.08999999999997</v>
+      </c>
+      <c r="C24">
+        <v>284.14</v>
+      </c>
+      <c r="D24">
+        <v>303.08999999999997</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>2179.6</v>
+      </c>
+      <c r="B25">
+        <v>337.82</v>
+      </c>
+      <c r="C25">
+        <v>320.23</v>
+      </c>
+      <c r="D25">
+        <v>337.82</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>2374</v>
+      </c>
+      <c r="B26">
+        <v>373.55</v>
+      </c>
+      <c r="C26">
+        <v>357.12</v>
+      </c>
+      <c r="D26">
+        <v>373.55</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>2567.1999999999998</v>
+      </c>
+      <c r="B27">
+        <v>407.53</v>
+      </c>
+      <c r="C27">
+        <v>392.09</v>
+      </c>
+      <c r="D27">
+        <v>407.53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>2756.5</v>
+      </c>
+      <c r="B28">
+        <v>439.28</v>
+      </c>
+      <c r="C28">
+        <v>424.71</v>
+      </c>
+      <c r="D28">
+        <v>439.28</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>2945.7</v>
+      </c>
+      <c r="B29">
+        <v>469.51</v>
+      </c>
+      <c r="C29">
+        <v>455.69</v>
+      </c>
+      <c r="D29">
+        <v>469.51</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>3134.9</v>
+      </c>
+      <c r="B30">
+        <v>498.24</v>
+      </c>
+      <c r="C30">
+        <v>485.07</v>
+      </c>
+      <c r="D30">
+        <v>498.24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>3324.1</v>
+      </c>
+      <c r="B31">
+        <v>525.52</v>
+      </c>
+      <c r="C31">
+        <v>512.94000000000005</v>
+      </c>
+      <c r="D31">
+        <v>525.52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>3513.3</v>
+      </c>
+      <c r="B32">
+        <v>551.42999999999995</v>
+      </c>
+      <c r="C32">
+        <v>539.37</v>
+      </c>
+      <c r="D32">
+        <v>551.42999999999995</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>3702.5</v>
+      </c>
+      <c r="B33">
+        <v>576.02</v>
+      </c>
+      <c r="C33">
+        <v>564.44000000000005</v>
+      </c>
+      <c r="D33">
+        <v>576.02</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>3891.7</v>
+      </c>
+      <c r="B34">
+        <v>599.36</v>
+      </c>
+      <c r="C34">
+        <v>588.23</v>
+      </c>
+      <c r="D34">
+        <v>599.36</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>4081</v>
+      </c>
+      <c r="B35">
+        <v>621.42999999999995</v>
+      </c>
+      <c r="C35">
+        <v>610.78</v>
+      </c>
+      <c r="D35">
+        <v>621.42999999999995</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>4270.2</v>
+      </c>
+      <c r="B36">
+        <v>642.19000000000005</v>
+      </c>
+      <c r="C36">
+        <v>632.03</v>
+      </c>
+      <c r="D36">
+        <v>642.19000000000005</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>4459.3999999999996</v>
+      </c>
+      <c r="B37">
+        <v>661.57</v>
+      </c>
+      <c r="C37">
+        <v>651.94000000000005</v>
+      </c>
+      <c r="D37">
+        <v>661.57</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>4648.6000000000004</v>
+      </c>
+      <c r="B38">
+        <v>679.46</v>
+      </c>
+      <c r="C38">
+        <v>670.42</v>
+      </c>
+      <c r="D38">
+        <v>679.46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>4837.8</v>
+      </c>
+      <c r="B39">
+        <v>695.64</v>
+      </c>
+      <c r="C39">
+        <v>687.32</v>
+      </c>
+      <c r="D39">
+        <v>695.64</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>5027</v>
+      </c>
+      <c r="B40">
+        <v>709.7</v>
+      </c>
+      <c r="C40">
+        <v>702.38</v>
+      </c>
+      <c r="D40">
+        <v>709.7</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>5216.2</v>
+      </c>
+      <c r="B41">
+        <v>720.68</v>
+      </c>
+      <c r="C41">
+        <v>714.81</v>
+      </c>
+      <c r="D41">
+        <v>720.68</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>5405.5</v>
+      </c>
+      <c r="B42">
+        <v>727.95</v>
+      </c>
+      <c r="C42">
+        <v>723.36</v>
+      </c>
+      <c r="D42">
+        <v>727.95</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>5594.7</v>
+      </c>
+      <c r="B43">
+        <v>732.61</v>
+      </c>
+      <c r="C43">
+        <v>729.85</v>
+      </c>
+      <c r="D43">
+        <v>732.61</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>5783.9</v>
+      </c>
+      <c r="B44">
+        <v>738.12</v>
+      </c>
+      <c r="C44">
+        <v>733.9</v>
+      </c>
+      <c r="D44">
+        <v>738.12</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>5973.1</v>
+      </c>
+      <c r="B45">
+        <v>746.99</v>
+      </c>
+      <c r="C45">
+        <v>738.4</v>
+      </c>
+      <c r="D45">
+        <v>746.99</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>6122</v>
+      </c>
+      <c r="B46">
+        <v>755.96</v>
+      </c>
+      <c r="C46">
+        <v>744.47</v>
+      </c>
+      <c r="D46">
+        <v>755.96</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>6270.7</v>
+      </c>
+      <c r="B47">
+        <v>766.48</v>
+      </c>
+      <c r="C47">
+        <v>754.41</v>
+      </c>
+      <c r="D47">
+        <v>766.48</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>6394.6</v>
+      </c>
+      <c r="B48">
+        <v>776.03</v>
+      </c>
+      <c r="C48">
+        <v>764.63</v>
+      </c>
+      <c r="D48">
+        <v>776.03</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>6504.6</v>
+      </c>
+      <c r="B49">
+        <v>784.94</v>
+      </c>
+      <c r="C49">
+        <v>774.55</v>
+      </c>
+      <c r="D49">
+        <v>784.94</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>6614.5</v>
+      </c>
+      <c r="B50">
+        <v>794.09</v>
+      </c>
+      <c r="C50">
+        <v>784.72</v>
+      </c>
+      <c r="D50">
+        <v>794.09</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>6710.5</v>
+      </c>
+      <c r="B51">
+        <v>801.8</v>
+      </c>
+      <c r="C51">
+        <v>792.69</v>
+      </c>
+      <c r="D51">
+        <v>801.8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>6806.5</v>
+      </c>
+      <c r="B52">
+        <v>809.92</v>
+      </c>
+      <c r="C52">
+        <v>801.71</v>
+      </c>
+      <c r="D52">
+        <v>809.92</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>6888</v>
+      </c>
+      <c r="B53">
+        <v>816.55</v>
+      </c>
+      <c r="C53">
+        <v>808.56</v>
+      </c>
+      <c r="D53">
+        <v>816.55</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>6969.5</v>
+      </c>
+      <c r="B54">
+        <v>823.1</v>
+      </c>
+      <c r="C54">
+        <v>815.3</v>
+      </c>
+      <c r="D54">
+        <v>823.1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>7053.8</v>
+      </c>
+      <c r="B55">
+        <v>829.77</v>
+      </c>
+      <c r="C55">
+        <v>822.12</v>
+      </c>
+      <c r="D55">
+        <v>829.77</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>7135.7</v>
+      </c>
+      <c r="B56">
+        <v>836.17</v>
+      </c>
+      <c r="C56">
+        <v>828.71</v>
+      </c>
+      <c r="D56">
+        <v>836.17</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>7214.5</v>
+      </c>
+      <c r="B57">
+        <v>842.27</v>
+      </c>
+      <c r="C57">
+        <v>835.02</v>
+      </c>
+      <c r="D57">
+        <v>842.27</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>7293.3</v>
+      </c>
+      <c r="B58">
+        <v>848.29</v>
+      </c>
+      <c r="C58">
+        <v>841.24</v>
+      </c>
+      <c r="D58">
+        <v>848.29</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>7372.1</v>
+      </c>
+      <c r="B59">
+        <v>854.21</v>
+      </c>
+      <c r="C59">
+        <v>847.35</v>
+      </c>
+      <c r="D59">
+        <v>854.21</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>7450.9</v>
+      </c>
+      <c r="B60">
+        <v>860.04</v>
+      </c>
+      <c r="C60">
+        <v>853.35</v>
+      </c>
+      <c r="D60">
+        <v>860.04</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>7529.8</v>
+      </c>
+      <c r="B61">
+        <v>865.77</v>
+      </c>
+      <c r="C61">
+        <v>859.24</v>
+      </c>
+      <c r="D61">
+        <v>865.77</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>7608.6</v>
+      </c>
+      <c r="B62">
+        <v>871.4</v>
+      </c>
+      <c r="C62">
+        <v>865.03</v>
+      </c>
+      <c r="D62">
+        <v>871.4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>7687.4</v>
+      </c>
+      <c r="B63">
+        <v>876.92</v>
+      </c>
+      <c r="C63">
+        <v>870.7</v>
+      </c>
+      <c r="D63">
+        <v>876.92</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>7766.2</v>
+      </c>
+      <c r="B64">
+        <v>882.33</v>
+      </c>
+      <c r="C64">
+        <v>876.27</v>
+      </c>
+      <c r="D64">
+        <v>882.33</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>7845.1</v>
+      </c>
+      <c r="B65">
+        <v>887.65</v>
+      </c>
+      <c r="C65">
+        <v>881.72</v>
+      </c>
+      <c r="D65">
+        <v>887.65</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>7923.9</v>
+      </c>
+      <c r="B66">
+        <v>892.86</v>
+      </c>
+      <c r="C66">
+        <v>887.07</v>
+      </c>
+      <c r="D66">
+        <v>892.87</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>8002.7</v>
+      </c>
+      <c r="B67">
+        <v>897.97</v>
+      </c>
+      <c r="C67">
+        <v>892.31</v>
+      </c>
+      <c r="D67">
+        <v>897.97</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>8081.5</v>
+      </c>
+      <c r="B68">
+        <v>902.98</v>
+      </c>
+      <c r="C68">
+        <v>897.45</v>
+      </c>
+      <c r="D68">
+        <v>902.98</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>8160.3</v>
+      </c>
+      <c r="B69">
+        <v>907.87</v>
+      </c>
+      <c r="C69">
+        <v>902.48</v>
+      </c>
+      <c r="D69">
+        <v>907.87</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>8239.2000000000007</v>
+      </c>
+      <c r="B70">
+        <v>912.66</v>
+      </c>
+      <c r="C70">
+        <v>907.39</v>
+      </c>
+      <c r="D70">
+        <v>912.66</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>8318</v>
+      </c>
+      <c r="B71">
+        <v>917.34</v>
+      </c>
+      <c r="C71">
+        <v>912.19</v>
+      </c>
+      <c r="D71">
+        <v>917.34</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>8396.7999999999993</v>
+      </c>
+      <c r="B72">
+        <v>921.91</v>
+      </c>
+      <c r="C72">
+        <v>916.88</v>
+      </c>
+      <c r="D72">
+        <v>921.91</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>8475.6</v>
+      </c>
+      <c r="B73">
+        <v>926.39</v>
+      </c>
+      <c r="C73">
+        <v>921.47</v>
+      </c>
+      <c r="D73">
+        <v>926.39</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>8554.4</v>
+      </c>
+      <c r="B74">
+        <v>930.77</v>
+      </c>
+      <c r="C74">
+        <v>925.95</v>
+      </c>
+      <c r="D74">
+        <v>930.77</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>8633.2999999999993</v>
+      </c>
+      <c r="B75">
+        <v>935.05</v>
+      </c>
+      <c r="C75">
+        <v>930.34</v>
+      </c>
+      <c r="D75">
+        <v>935.05</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>8712.1</v>
+      </c>
+      <c r="B76">
+        <v>939.24</v>
+      </c>
+      <c r="C76">
+        <v>934.64</v>
+      </c>
+      <c r="D76">
+        <v>939.24</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>8790.9</v>
+      </c>
+      <c r="B77">
+        <v>943.35</v>
+      </c>
+      <c r="C77">
+        <v>938.84</v>
+      </c>
+      <c r="D77">
+        <v>943.35</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>8869.7000000000007</v>
+      </c>
+      <c r="B78">
+        <v>947.36</v>
+      </c>
+      <c r="C78">
+        <v>942.95</v>
+      </c>
+      <c r="D78">
+        <v>947.36</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>8948.5</v>
+      </c>
+      <c r="B79">
+        <v>951.3</v>
+      </c>
+      <c r="C79">
+        <v>946.98</v>
+      </c>
+      <c r="D79">
+        <v>951.3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>9000</v>
+      </c>
+      <c r="B80">
+        <v>953.96</v>
+      </c>
+      <c r="C80">
+        <v>949.88</v>
+      </c>
+      <c r="D80">
+        <v>953.96</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>